<commit_message>
3 file mẫu Excel
</commit_message>
<xml_diff>
--- a/data/TEMPLATE_CHINESE.xlsx
+++ b/data/TEMPLATE_CHINESE.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chinese H3" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chinese Basic" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +28,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -40,12 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="00366092"/>
+        <bgColor rgb="00366092"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -53,25 +53,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,184 +427,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>STT</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Meaning</t>
+          <t>word</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Example EN</t>
+          <t>meaning</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Example VI</t>
+          <t>example_zh</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>example_vi</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>你好</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>xin chào</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>你好，我是李明。</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Xin chào, tôi là Lý Minh.</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>你好，你好吗？</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Xin chào, bạn khỏe không?</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>谢谢</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>cảm ơn</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>谢谢你的帮助。</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Cảm ơn bạn đã giúp tôi.</t>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>非常感谢你</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Cảm ơn bạn rất nhiều</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>再见</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>tạm biệt</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>再见，明天见。</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Tạm biệt, ngày mai gặp lại.</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>再见，回头见</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Tạm biệt, hẹn gặp lại</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>请</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>làm ơn</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>请帮帮我</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Làm ơn giúp tôi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>对不起</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>xin lỗi</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>对不起，我迟到了。</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Xin lỗi, tôi đến muộn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>对不起，我错了</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Xin lỗi, tôi sai rồi</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>có/phải</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>是的，我同意</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Vâng, tôi đồng ý</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>不是</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>không phải</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>不是，我不同意</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Không, tôi không đồng ý</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>早上好</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>chào buổi sáng</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>早上好，大家</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Chào buổi sáng mọi người</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>晚安</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>chúc ngủ ngon</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>晚安，做个好梦</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Chúc ngủ ngon, mơ đẹp</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>怎么</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>như thế nào</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>你怎么做的？</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Bạn làm như thế nào?</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>